<commit_message>
feat: implement stock monitor logic and add initial configuration and market data files
</commit_message>
<xml_diff>
--- a/outputs/monitor_xlsx/20260407.xlsx
+++ b/outputs/monitor_xlsx/20260407.xlsx
@@ -536,14 +536,18 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>32572.43</t>
+          <t>33229.82</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.82%</t>
-        </is>
-      </c>
+          <t>+2.02%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -558,14 +562,18 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>317.9</t>
+          <t>325.61</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.02%</t>
-        </is>
-      </c>
+          <t>+2.43%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -588,6 +596,10 @@
           <t>+2.01%</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -610,6 +622,10 @@
           <t>+0.12%</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -624,14 +640,18 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>4837.9$</t>
+          <t>4657.1$</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+3.89%</t>
-        </is>
-      </c>
+          <t>+0.01%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -654,6 +674,10 @@
           <t>-0.17%</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -676,6 +700,10 @@
           <t>+1.11%</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -698,6 +726,10 @@
           <t>+6.66%</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -712,14 +744,18 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>97.43$</t>
+          <t>112.95$</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-13.33%</t>
-        </is>
-      </c>
+          <t>+0.48%</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -734,17 +770,18 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>100.97億</t>
-        </is>
-      </c>
+          <t>100.75億</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>-392.96億</t>
+          <t>-295.38億</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>-1964.82億</t>
+          <t>-1476.9億</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -771,19 +808,22 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>43.57億</t>
-        </is>
-      </c>
+          <t>24.52億</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>49.57億</t>
+          <t>41.43億</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>247.85億</t>
-        </is>
-      </c>
+          <t>207.17億</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -798,14 +838,18 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>139.18%</t>
-        </is>
-      </c>
+          <t>109.19%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>130.26%</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -820,9 +864,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>214.86億</t>
-        </is>
-      </c>
+          <t>195.6億</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -840,11 +889,15 @@
           <t>4789口</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>8568口</t>
-        </is>
-      </c>
+          <t>7958口</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -862,24 +915,25 @@
           <t>-38.64億</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>8.05億</t>
+          <t>6.86億</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>40.24億</t>
+          <t>34.29億</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>-7.94億</t>
+          <t>-7.68億</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>-158.74億</t>
+          <t>-153.59億</t>
         </is>
       </c>
     </row>
@@ -926,7 +980,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>-392.96億</t>
+          <t>-295.38億</t>
         </is>
       </c>
     </row>
@@ -938,7 +992,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>-1964.82億</t>
+          <t>-1476.9億</t>
         </is>
       </c>
     </row>
@@ -966,6 +1020,10 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -974,7 +1032,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>49.57億</t>
+          <t>41.43億</t>
         </is>
       </c>
     </row>
@@ -986,7 +1044,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>247.85億</t>
+          <t>207.17億</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1063,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8.05億</t>
+          <t>6.86億</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1075,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>40.24億</t>
+          <t>34.29億</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1087,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>-7.94億</t>
+          <t>-7.68億</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1099,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>-158.74億</t>
+          <t>-153.59億</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1130,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>8568口</t>
+          <t>7958口</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W18"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1122,7 +1180,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1269,13 +1326,13 @@
         <v>-2592</v>
       </c>
       <c r="H4" t="n">
-        <v>-273790</v>
+        <v>-98910</v>
       </c>
       <c r="I4" t="n">
         <v>2700</v>
       </c>
       <c r="J4" t="n">
-        <v>3500</v>
+        <v>-1400</v>
       </c>
       <c r="K4" t="n">
         <v>15143</v>
@@ -1284,17 +1341,14 @@
         <v>12650</v>
       </c>
       <c r="M4" t="n">
-        <v>69854</v>
+        <v>56334</v>
       </c>
       <c r="N4" t="n">
         <v>-4627553</v>
       </c>
-      <c r="O4" t="n">
-        <v>1.58</v>
-      </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>主力積極賣出</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
@@ -1332,13 +1386,13 @@
         <v>87</v>
       </c>
       <c r="H5" t="n">
-        <v>1921</v>
+        <v>2515</v>
       </c>
       <c r="I5" t="n">
         <v>-129</v>
       </c>
       <c r="J5" t="n">
-        <v>-1680</v>
+        <v>-738</v>
       </c>
       <c r="K5" t="n">
         <v>80</v>
@@ -1347,14 +1401,11 @@
         <v>2679</v>
       </c>
       <c r="M5" t="n">
-        <v>13692</v>
+        <v>10851</v>
       </c>
       <c r="N5" t="n">
         <v>-78961</v>
       </c>
-      <c r="O5" t="n">
-        <v>-4.15</v>
-      </c>
       <c r="P5" t="inlineStr">
         <is>
           <t>中性</t>
@@ -1395,13 +1446,13 @@
         <v>3601</v>
       </c>
       <c r="H6" t="n">
-        <v>-10473</v>
+        <v>-5186</v>
       </c>
       <c r="I6" t="n">
         <v>-14</v>
       </c>
       <c r="J6" t="n">
-        <v>1212</v>
+        <v>746</v>
       </c>
       <c r="K6" t="n">
         <v>166</v>
@@ -1410,14 +1461,11 @@
         <v>5009</v>
       </c>
       <c r="M6" t="n">
-        <v>27472</v>
+        <v>21676</v>
       </c>
       <c r="N6" t="n">
         <v>-649316</v>
       </c>
-      <c r="O6" t="n">
-        <v>4.05</v>
-      </c>
       <c r="P6" t="inlineStr">
         <is>
           <t>偏空</t>
@@ -1458,13 +1506,13 @@
         <v>5880</v>
       </c>
       <c r="H7" t="n">
-        <v>-50738</v>
+        <v>-14256</v>
       </c>
       <c r="I7" t="n">
         <v>421</v>
       </c>
       <c r="J7" t="n">
-        <v>2801</v>
+        <v>2054</v>
       </c>
       <c r="K7" t="n">
         <v>312</v>
@@ -1473,14 +1521,11 @@
         <v>26000</v>
       </c>
       <c r="M7" t="n">
-        <v>132639</v>
+        <v>106254</v>
       </c>
       <c r="N7" t="n">
         <v>-6483112</v>
       </c>
-      <c r="O7" t="n">
-        <v>3.05</v>
-      </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>偏空</t>
@@ -1521,13 +1566,13 @@
         <v>-788</v>
       </c>
       <c r="H8" t="n">
-        <v>-1784</v>
+        <v>-768</v>
       </c>
       <c r="I8" t="n">
         <v>-25</v>
       </c>
       <c r="J8" t="n">
-        <v>1959</v>
+        <v>671</v>
       </c>
       <c r="K8" t="n">
         <v>99</v>
@@ -1536,17 +1581,14 @@
         <v>1914</v>
       </c>
       <c r="M8" t="n">
-        <v>10528</v>
+        <v>8238</v>
       </c>
       <c r="N8" t="n">
         <v>-140279</v>
       </c>
-      <c r="O8" t="n">
-        <v>0.31</v>
-      </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>🔴偏空 (法人齊賣)</t>
         </is>
       </c>
       <c r="W8" t="inlineStr">
@@ -1566,50 +1608,47 @@
           <t>致茂</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>上市</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>1570</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="E9" s="6" t="n">
         <v>2.28</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="F9" t="n">
         <v>3326</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="G9" s="6" t="n">
         <v>-526</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>-234</v>
-      </c>
       <c r="H9" t="n">
+        <v>334</v>
+      </c>
+      <c r="I9" t="n">
         <v>89</v>
       </c>
-      <c r="I9" t="n">
-        <v>441</v>
-      </c>
       <c r="J9" t="n">
+        <v>-117</v>
+      </c>
+      <c r="K9" t="n">
         <v>36</v>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>2088</v>
       </c>
-      <c r="L9" t="n">
-        <v>11066</v>
-      </c>
       <c r="M9" t="n">
+        <v>8978</v>
+      </c>
+      <c r="N9" t="n">
         <v>-106310</v>
       </c>
-      <c r="N9" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="W9" t="inlineStr">
@@ -1647,13 +1686,13 @@
         <v>-39</v>
       </c>
       <c r="H10" t="n">
-        <v>-955</v>
+        <v>9</v>
       </c>
       <c r="I10" t="n">
         <v>71</v>
       </c>
       <c r="J10" t="n">
-        <v>557</v>
+        <v>295</v>
       </c>
       <c r="K10" t="n">
         <v>78</v>
@@ -1662,17 +1701,14 @@
         <v>1847</v>
       </c>
       <c r="M10" t="n">
-        <v>9263</v>
+        <v>7377</v>
       </c>
       <c r="N10" t="n">
         <v>-89560</v>
       </c>
-      <c r="O10" t="n">
-        <v>3.48</v>
-      </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>偏多</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
@@ -1684,12 +1720,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6442</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>光聖</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1698,44 +1734,41 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2095</v>
+        <v>7100</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>4.75</v>
+        <v>7.49</v>
       </c>
       <c r="F11" t="n">
-        <v>2764</v>
+        <v>237</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>343</v>
+        <v>56</v>
       </c>
       <c r="H11" t="n">
-        <v>-674</v>
+        <v>100</v>
       </c>
       <c r="I11" t="n">
-        <v>-18</v>
+        <v>-41</v>
       </c>
       <c r="J11" t="n">
-        <v>255</v>
+        <v>-142</v>
       </c>
       <c r="K11" t="n">
-        <v>57</v>
+        <v>10</v>
       </c>
       <c r="L11" t="n">
-        <v>3817</v>
+        <v>328</v>
       </c>
       <c r="M11" t="n">
-        <v>19626</v>
+        <v>1242</v>
       </c>
       <c r="N11" t="n">
-        <v>-19417</v>
-      </c>
-      <c r="O11" t="n">
-        <v>3.15</v>
+        <v>-8989</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
@@ -1747,54 +1780,51 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>3081</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>穎崴</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>7100</v>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>7.49</v>
+          <t>聯亞</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>上櫃</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2105</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>237</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>56</v>
-      </c>
-      <c r="G12" s="7" t="n">
-        <v>257</v>
+        <v>3.19</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2931</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>-401</v>
       </c>
       <c r="H12" t="n">
-        <v>-41</v>
+        <v>-23</v>
       </c>
       <c r="I12" t="n">
-        <v>-370</v>
+        <v>83</v>
       </c>
       <c r="J12" t="n">
-        <v>10</v>
+        <v>298</v>
       </c>
       <c r="K12" t="n">
-        <v>328</v>
+        <v>-49</v>
       </c>
       <c r="L12" t="n">
-        <v>1570</v>
+        <v>198</v>
       </c>
       <c r="M12" t="n">
-        <v>-8989</v>
+        <v>-96</v>
       </c>
       <c r="N12" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>中性</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
@@ -1810,12 +1840,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3081</t>
+          <t>4979</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>聯亞</t>
+          <t>華星光</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1824,44 +1854,38 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2005</v>
+        <v>429</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>9.859999999999999</v>
+        <v>1.78</v>
       </c>
       <c r="F13" t="n">
-        <v>3109</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>-401</v>
+        <v>2073</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>107</v>
       </c>
       <c r="H13" t="n">
-        <v>-12</v>
-      </c>
-      <c r="I13" t="n">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="J13" t="n">
-        <v>946</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>-49</v>
+        <v>25</v>
       </c>
       <c r="L13" t="n">
-        <v>198</v>
+        <v>-54</v>
       </c>
       <c r="M13" t="n">
-        <v>76</v>
+        <v>-1238</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
       </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>主力積極買進</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
@@ -1873,12 +1897,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4979</t>
+          <t>6187</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>華星光</t>
+          <t>萬潤</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1887,41 +1911,38 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>404.5</v>
-      </c>
-      <c r="E14" s="6" t="n">
-        <v>5.34</v>
+        <v>886</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>-9.59</v>
       </c>
       <c r="F14" t="n">
-        <v>1185</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>107</v>
+        <v>972</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>-49</v>
       </c>
       <c r="H14" t="n">
-        <v>-200</v>
+        <v>369</v>
       </c>
       <c r="J14" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>25</v>
+        <v>-0</v>
       </c>
       <c r="L14" t="n">
-        <v>-54</v>
+        <v>-23</v>
       </c>
       <c r="M14" t="n">
-        <v>-1627</v>
+        <v>-486</v>
       </c>
       <c r="N14" t="n">
         <v>0</v>
       </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>偏空</t>
+          <t>主力積極買進</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
@@ -1933,12 +1954,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6187</t>
+          <t>6640</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>萬潤</t>
+          <t>均華</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1947,224 +1968,41 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>920</v>
+        <v>1525</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>2.79</v>
+        <v>4.45</v>
       </c>
       <c r="F15" t="n">
-        <v>583</v>
+        <v>962</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>-49</v>
+        <v>-18</v>
       </c>
       <c r="H15" t="n">
-        <v>1463</v>
+        <v>-65</v>
       </c>
       <c r="J15" t="n">
-        <v>346</v>
+        <v>118</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="L15" t="n">
-        <v>-23</v>
+        <v>-22</v>
       </c>
       <c r="M15" t="n">
-        <v>-572</v>
+        <v>-136</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>主力積極買進</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>6640</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>均華</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>上櫃</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>1330</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>-3.27</v>
-      </c>
-      <c r="F16" t="n">
-        <v>473</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>-18</v>
-      </c>
-      <c r="H16" t="n">
-        <v>-59</v>
-      </c>
-      <c r="J16" t="n">
-        <v>118</v>
-      </c>
-      <c r="K16" t="n">
-        <v>19</v>
-      </c>
-      <c r="L16" t="n">
-        <v>-22</v>
-      </c>
-      <c r="M16" t="n">
-        <v>28</v>
-      </c>
-      <c r="N16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>偏空</t>
-        </is>
-      </c>
-      <c r="W16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>1305</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>華夏</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>上市</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>-1.95</v>
-      </c>
-      <c r="F17" t="n">
-        <v>24067</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>-969</v>
-      </c>
-      <c r="H17" t="n">
-        <v>-8376</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>28</v>
-      </c>
-      <c r="L17" t="n">
-        <v>9686</v>
-      </c>
-      <c r="M17" t="n">
-        <v>44388</v>
-      </c>
-      <c r="N17" t="n">
-        <v>-145009</v>
-      </c>
-      <c r="O17" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>主力積極賣出</t>
-        </is>
-      </c>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>1309</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>台達化</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>上市</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>2.12</v>
-      </c>
-      <c r="F18" t="n">
-        <v>84038</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>-708</v>
-      </c>
-      <c r="H18" t="n">
-        <v>716</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" t="n">
-        <v>377</v>
-      </c>
-      <c r="L18" t="n">
-        <v>11156</v>
-      </c>
-      <c r="M18" t="n">
-        <v>46981</v>
-      </c>
-      <c r="N18" t="n">
-        <v>-97545</v>
-      </c>
-      <c r="O18" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="P18" t="inlineStr">
-        <is>
-          <t>偏多</t>
-        </is>
-      </c>
-      <c r="W18" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>